<commit_message>
Merge develop into student5
</commit_message>
<xml_diff>
--- a/Planning-Template.xlsx
+++ b/Planning-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franr\OneDrive\Escritorio\informatica_us\asignaturas\DP2\ent\Workspace-26\Projects\Acme-Starters-C\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E258BD7-A18C-4E3F-99CF-DB18BA672F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BED9D66B-D0DD-421B-9137-D405D31496CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" activeTab="2" xr2:uid="{683E09B8-1D94-4905-B116-9D998A46AAA3}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="95">
   <si>
     <t xml:space="preserve">  Enter configuration data in these cells</t>
   </si>
@@ -338,6 +338,12 @@
   </si>
   <si>
     <t>T0002/D</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>T0004/D</t>
   </si>
 </sst>
 </file>
@@ -711,6 +717,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -728,9 +737,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,118 +1376,118 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="55" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="53"/>
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54"/>
+      <c r="F7" s="54"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="54"/>
+      <c r="I7" s="54"/>
+      <c r="J7" s="54"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B8" s="53"/>
-      <c r="C8" s="53"/>
-      <c r="D8" s="53"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="53"/>
-      <c r="G8" s="53"/>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="53"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="54"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="53"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="53"/>
-      <c r="G9" s="53"/>
-      <c r="H9" s="53"/>
-      <c r="I9" s="53"/>
-      <c r="J9" s="53"/>
+      <c r="B9" s="54"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
+      <c r="J9" s="54"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="53"/>
-      <c r="G10" s="53"/>
-      <c r="H10" s="53"/>
-      <c r="I10" s="53"/>
-      <c r="J10" s="53"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="54"/>
+      <c r="G10" s="54"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
+      <c r="J10" s="54"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="53"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="53"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
-      <c r="I11" s="53"/>
-      <c r="J11" s="53"/>
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="54"/>
+      <c r="I11" s="54"/>
+      <c r="J11" s="54"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
-      <c r="D12" s="53"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="53"/>
-      <c r="G12" s="53"/>
-      <c r="H12" s="53"/>
-      <c r="I12" s="53"/>
-      <c r="J12" s="53"/>
+      <c r="B12" s="54"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="54"/>
+      <c r="G12" s="54"/>
+      <c r="H12" s="54"/>
+      <c r="I12" s="54"/>
+      <c r="J12" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1499,17 +1505,17 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B3" s="2"/>
@@ -1523,39 +1529,39 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="53"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="1"/>
@@ -1583,29 +1589,29 @@
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9" s="4"/>
-      <c r="C9" s="55" t="s">
+      <c r="C9" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
+      <c r="J9" s="56"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B10" s="48"/>
-      <c r="C10" s="55" t="s">
+      <c r="C10" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="55"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="55"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="56"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B11" s="49"/>
@@ -1622,16 +1628,16 @@
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
-      <c r="C12" s="55" t="s">
+      <c r="C12" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="55"/>
+      <c r="D12" s="56"/>
+      <c r="E12" s="56"/>
+      <c r="F12" s="56"/>
+      <c r="G12" s="56"/>
+      <c r="H12" s="56"/>
+      <c r="I12" s="56"/>
+      <c r="J12" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1655,40 +1661,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C2" s="54" t="s">
+      <c r="C2" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="55"/>
     </row>
     <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
-      <c r="K4" s="52"/>
-      <c r="L4" s="52"/>
-      <c r="M4" s="52"/>
-      <c r="N4" s="52"/>
-      <c r="O4" s="52"/>
-      <c r="P4" s="52"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="53"/>
+      <c r="P4" s="53"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C5" s="5"/>
@@ -1707,7 +1713,7 @@
       <c r="P5" s="5"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="57" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="10" t="s">
@@ -1730,7 +1736,7 @@
       <c r="P6" s="5"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C7" s="56"/>
+      <c r="C7" s="57"/>
       <c r="D7" s="11" t="s">
         <v>69</v>
       </c>
@@ -1748,19 +1754,19 @@
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="57" t="s">
+      <c r="I9" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="57"/>
+      <c r="J9" s="58"/>
       <c r="K9" s="7"/>
-      <c r="L9" s="57" t="s">
+      <c r="L9" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="M9" s="57"/>
-      <c r="N9" s="57" t="s">
+      <c r="M9" s="58"/>
+      <c r="N9" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="O9" s="57"/>
+      <c r="O9" s="58"/>
       <c r="P9" s="7"/>
     </row>
     <row r="10" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1822,7 +1828,7 @@
         <v>63</v>
       </c>
       <c r="E11" s="42" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F11" s="42" t="s">
         <v>27</v>
@@ -1910,7 +1916,7 @@
         <v>61</v>
       </c>
       <c r="E13" s="42" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F13" s="42" t="s">
         <v>25</v>
@@ -1929,7 +1935,7 @@
       </c>
       <c r="K13" s="44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>Ongoing</v>
+        <v>Completed</v>
       </c>
       <c r="L13" s="46"/>
       <c r="M13" s="46"/>
@@ -1949,18 +1955,27 @@
       </c>
       <c r="C14" s="41" t="str">
         <f>IF(ISBLANK(D14), "", _xlfn.CONCAT("T", TEXT(B14, "0000"), "/", VLOOKUP(D14, Internal!$B$35:C$39, 2, FALSE), IF(OR(D14="QA", D14="Revision"), _xlfn.CONCAT("/", H14), "")))</f>
-        <v/>
-      </c>
-      <c r="D14" s="43"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="42"/>
+        <v>T0004/D</v>
+      </c>
+      <c r="D14" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="42" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="42" t="s">
+        <v>92</v>
+      </c>
       <c r="I14" s="45"/>
       <c r="J14" s="45"/>
-      <c r="K14" s="44" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
+      <c r="K14" s="44" t="s">
+        <v>93</v>
       </c>
       <c r="L14" s="46"/>
       <c r="M14" s="46"/>
@@ -1980,18 +1995,30 @@
       </c>
       <c r="C15" s="41" t="str">
         <f>IF(ISBLANK(D15), "", _xlfn.CONCAT("T", TEXT(B15, "0000"), "/", VLOOKUP(D15, Internal!$B$35:C$39, 2, FALSE), IF(OR(D15="QA", D15="Revision"), _xlfn.CONCAT("/", H15), "")))</f>
-        <v/>
-      </c>
-      <c r="D15" s="43"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="43"/>
+        <v>T0005/M</v>
+      </c>
+      <c r="D15" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="43" t="s">
+        <v>36</v>
+      </c>
       <c r="H15" s="42"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="45"/>
+      <c r="I15" s="45">
+        <v>46063.479166666664</v>
+      </c>
+      <c r="J15" s="45">
+        <v>46063.5625</v>
+      </c>
       <c r="K15" s="44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>Completed</v>
       </c>
       <c r="L15" s="46"/>
       <c r="M15" s="46"/>
@@ -2011,13 +2038,23 @@
       </c>
       <c r="C16" s="41" t="str">
         <f>IF(ISBLANK(D16), "", _xlfn.CONCAT("T", TEXT(B16, "0000"), "/", VLOOKUP(D16, Internal!$B$35:C$39, 2, FALSE), IF(OR(D16="QA", D16="Revision"), _xlfn.CONCAT("/", H16), "")))</f>
-        <v/>
-      </c>
-      <c r="D16" s="43"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="42"/>
+        <v>T0006/M</v>
+      </c>
+      <c r="D16" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="42" t="s">
+        <v>94</v>
+      </c>
       <c r="I16" s="45"/>
       <c r="J16" s="45"/>
       <c r="K16" s="44" t="str">
@@ -5045,40 +5082,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C2" s="54" t="s">
+      <c r="C2" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="55"/>
     </row>
     <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
-      <c r="K4" s="52"/>
-      <c r="L4" s="52"/>
-      <c r="M4" s="52"/>
-      <c r="N4" s="52"/>
-      <c r="O4" s="52"/>
-      <c r="P4" s="52"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="53"/>
+      <c r="P4" s="53"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C5" s="5"/>
@@ -5097,7 +5134,7 @@
       <c r="P5" s="5"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="57" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="10" t="s">
@@ -5120,7 +5157,7 @@
       <c r="P6" s="5"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C7" s="56"/>
+      <c r="C7" s="57"/>
       <c r="D7" s="11" t="s">
         <v>69</v>
       </c>
@@ -5138,19 +5175,19 @@
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="57" t="s">
+      <c r="I9" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="57"/>
+      <c r="J9" s="58"/>
       <c r="K9" s="7"/>
-      <c r="L9" s="57" t="s">
+      <c r="L9" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="M9" s="57"/>
-      <c r="N9" s="57" t="s">
+      <c r="M9" s="58"/>
+      <c r="N9" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="O9" s="57"/>
+      <c r="O9" s="58"/>
       <c r="P9" s="7"/>
     </row>
     <row r="10" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -8394,40 +8431,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C2" s="54" t="s">
+      <c r="C2" s="55" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="55"/>
     </row>
     <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
-      <c r="K4" s="52"/>
-      <c r="L4" s="52"/>
-      <c r="M4" s="52"/>
-      <c r="N4" s="52"/>
-      <c r="O4" s="52"/>
-      <c r="P4" s="52"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="53"/>
+      <c r="P4" s="53"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C5" s="5"/>
@@ -8446,7 +8483,7 @@
       <c r="P5" s="5"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="57" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="10" t="s">
@@ -8469,7 +8506,7 @@
       <c r="P6" s="5"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="C7" s="56"/>
+      <c r="C7" s="57"/>
       <c r="D7" s="11" t="s">
         <v>69</v>
       </c>
@@ -8487,19 +8524,19 @@
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="57" t="s">
+      <c r="I9" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="57"/>
+      <c r="J9" s="58"/>
       <c r="K9" s="7"/>
-      <c r="L9" s="57" t="s">
+      <c r="L9" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="M9" s="57"/>
-      <c r="N9" s="57" t="s">
+      <c r="M9" s="58"/>
+      <c r="N9" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="O9" s="57"/>
+      <c r="O9" s="58"/>
       <c r="P9" s="7"/>
     </row>
     <row r="10" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -11742,52 +11779,52 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="53"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="5"/>
@@ -11992,7 +12029,7 @@
       <c r="J22" s="12"/>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B23" s="58">
+      <c r="B23" s="52">
         <v>46062.354166666664</v>
       </c>
       <c r="C23" s="12"/>

</xml_diff>

<commit_message>
docs: reorganizar y añadir A
</commit_message>
<xml_diff>
--- a/Planning-Template.xlsx
+++ b/Planning-Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alvar\Desktop\DP2-2526\Workspace-26\Projects\Acme-Starters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franr\OneDrive\Escritorio\informatica_us\asignaturas\DP2\ent\Workspace-26\Projects\Acme-Starters-B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CC2C1CD-94BA-4120-82C1-850708545C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A258C7E-C0DA-46A2-AAD8-A6F2BD36B29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5340" yWindow="-16320" windowWidth="38640" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Copyright" sheetId="1" r:id="rId1"/>
@@ -46,8 +46,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="169">
   <si>
     <t>Copyright</t>
   </si>
@@ -537,15 +559,38 @@
   <si>
     <t>Redactar documento de Testing Report</t>
   </si>
+  <si>
+    <t>Escrbir requisitos elicitados en el analysis report</t>
+  </si>
+  <si>
+    <t>Definir tareas analizando API y posibilidades</t>
+  </si>
+  <si>
+    <t>T0002/M</t>
+  </si>
+  <si>
+    <t>Implementar conexión con jobicy</t>
+  </si>
+  <si>
+    <t>T0003/D</t>
+  </si>
+  <si>
+    <t>Comprobar funcionamiento correcto</t>
+  </si>
+  <si>
+    <t>Comprobar implementacion en follow up</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$EUR]\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy\ h:mm"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -954,9 +999,9 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="6" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1732,12 +1777,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:AMJ12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1024" width="9.109375" style="2"/>
+    <col min="1" max="1024" width="9.08984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B2" s="63" t="s">
         <v>0</v>
       </c>
@@ -1750,7 +1795,7 @@
       <c r="I2" s="63"/>
       <c r="J2" s="63"/>
     </row>
-    <row r="4" spans="2:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="64" t="s">
         <v>1</v>
       </c>
@@ -1763,7 +1808,7 @@
       <c r="I4" s="64"/>
       <c r="J4" s="64"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
       <c r="D5" s="64"/>
@@ -1774,7 +1819,7 @@
       <c r="I5" s="64"/>
       <c r="J5" s="64"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6" s="64"/>
       <c r="C6" s="64"/>
       <c r="D6" s="64"/>
@@ -1785,7 +1830,7 @@
       <c r="I6" s="64"/>
       <c r="J6" s="64"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="64"/>
       <c r="C7" s="64"/>
       <c r="D7" s="64"/>
@@ -1796,7 +1841,7 @@
       <c r="I7" s="64"/>
       <c r="J7" s="64"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8" s="64"/>
       <c r="C8" s="64"/>
       <c r="D8" s="64"/>
@@ -1807,7 +1852,7 @@
       <c r="I8" s="64"/>
       <c r="J8" s="64"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9" s="64"/>
       <c r="C9" s="64"/>
       <c r="D9" s="64"/>
@@ -1818,7 +1863,7 @@
       <c r="I9" s="64"/>
       <c r="J9" s="64"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B10" s="64"/>
       <c r="C10" s="64"/>
       <c r="D10" s="64"/>
@@ -1829,7 +1874,7 @@
       <c r="I10" s="64"/>
       <c r="J10" s="64"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B11" s="64"/>
       <c r="C11" s="64"/>
       <c r="D11" s="64"/>
@@ -1840,7 +1885,7 @@
       <c r="I11" s="64"/>
       <c r="J11" s="64"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B12" s="64"/>
       <c r="C12" s="64"/>
       <c r="D12" s="64"/>
@@ -1865,9 +1910,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:J12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B2" s="63" t="s">
         <v>2</v>
       </c>
@@ -1880,7 +1925,7 @@
       <c r="I2" s="63"/>
       <c r="J2" s="63"/>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B3" s="3"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -1891,7 +1936,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="64" t="s">
         <v>3</v>
       </c>
@@ -1904,7 +1949,7 @@
       <c r="I4" s="64"/>
       <c r="J4" s="64"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
       <c r="D5" s="64"/>
@@ -1915,7 +1960,7 @@
       <c r="I5" s="64"/>
       <c r="J5" s="64"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6" s="64"/>
       <c r="C6" s="64"/>
       <c r="D6" s="64"/>
@@ -1926,7 +1971,7 @@
       <c r="I6" s="64"/>
       <c r="J6" s="64"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -1937,7 +1982,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8" s="4"/>
       <c r="C8" s="2" t="s">
         <v>4</v>
@@ -1950,7 +1995,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9" s="5"/>
       <c r="C9" s="67" t="s">
         <v>5</v>
@@ -1963,7 +2008,7 @@
       <c r="I9" s="67"/>
       <c r="J9" s="67"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
       <c r="C10" s="67" t="s">
         <v>6</v>
@@ -1976,7 +2021,7 @@
       <c r="I10" s="67"/>
       <c r="J10" s="67"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B11" s="7"/>
       <c r="C11" s="1" t="s">
         <v>7</v>
@@ -1989,7 +2034,7 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B12" s="8"/>
       <c r="C12" s="67" t="s">
         <v>8</v>
@@ -2018,16 +2063,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:P110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="6" width="18.88671875" customWidth="1"/>
-    <col min="7" max="7" width="23.44140625" customWidth="1"/>
-    <col min="8" max="8" width="13.5546875" customWidth="1"/>
-    <col min="9" max="15" width="18.88671875" customWidth="1"/>
-    <col min="16" max="16" width="64.5546875" customWidth="1"/>
+    <col min="3" max="6" width="18.90625" customWidth="1"/>
+    <col min="7" max="7" width="23.453125" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" customWidth="1"/>
+    <col min="9" max="15" width="18.90625" customWidth="1"/>
+    <col min="16" max="16" width="64.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C2" s="63" t="s">
         <v>9</v>
       </c>
@@ -2045,7 +2090,7 @@
       <c r="O2" s="63"/>
       <c r="P2" s="63"/>
     </row>
-    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C4" s="64" t="s">
         <v>10</v>
       </c>
@@ -2063,7 +2108,7 @@
       <c r="O4" s="64"/>
       <c r="P4" s="64"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -2079,7 +2124,7 @@
       <c r="O5" s="9"/>
       <c r="P5" s="9"/>
     </row>
-    <row r="6" spans="2:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C6" s="65" t="s">
         <v>11</v>
       </c>
@@ -2102,7 +2147,7 @@
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C7" s="65"/>
       <c r="D7" s="12" t="s">
         <v>13</v>
@@ -2113,7 +2158,7 @@
       </c>
       <c r="J7" s="14"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B9" s="15"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
@@ -2136,7 +2181,7 @@
       <c r="O9" s="66"/>
       <c r="P9" s="16"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B10" s="53" t="s">
         <v>17</v>
       </c>
@@ -2183,7 +2228,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B11" s="20">
         <v>1</v>
       </c>
@@ -2232,7 +2277,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B12" s="20">
         <v>2</v>
       </c>
@@ -2281,7 +2326,7 @@
       </c>
       <c r="P12" s="22"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B13" s="20">
         <v>3</v>
       </c>
@@ -2332,7 +2377,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B14" s="20">
         <v>4</v>
       </c>
@@ -2382,7 +2427,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B15" s="20">
         <v>5</v>
       </c>
@@ -2431,7 +2476,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B16" s="20">
         <v>6</v>
       </c>
@@ -2482,7 +2527,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B17" s="20">
         <v>7</v>
       </c>
@@ -2533,7 +2578,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B18" s="20">
         <v>8</v>
       </c>
@@ -2584,7 +2629,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B19" s="20">
         <v>9</v>
       </c>
@@ -2635,7 +2680,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B20" s="20">
         <v>10</v>
       </c>
@@ -2686,7 +2731,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B21" s="20">
         <v>11</v>
       </c>
@@ -2737,7 +2782,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B22" s="20">
         <v>12</v>
       </c>
@@ -2788,7 +2833,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B23" s="20">
         <v>13</v>
       </c>
@@ -2837,7 +2882,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B24" s="20">
         <v>14</v>
       </c>
@@ -2888,7 +2933,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B25" s="20">
         <v>15</v>
       </c>
@@ -2939,7 +2984,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B26" s="20">
         <v>16</v>
       </c>
@@ -2987,7 +3032,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B27" s="20">
         <v>17</v>
       </c>
@@ -3036,7 +3081,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B28" s="20">
         <v>18</v>
       </c>
@@ -3085,7 +3130,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="20">
         <v>19</v>
       </c>
@@ -3134,7 +3179,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B30" s="20">
         <v>20</v>
       </c>
@@ -3183,7 +3228,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B31" s="20">
         <v>21</v>
       </c>
@@ -3232,7 +3277,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B32" s="20">
         <v>22</v>
       </c>
@@ -3281,7 +3326,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B33" s="20">
         <v>23</v>
       </c>
@@ -3330,7 +3375,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B34" s="20">
         <v>24</v>
       </c>
@@ -3379,7 +3424,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="35" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B35" s="20">
         <v>25</v>
       </c>
@@ -3427,7 +3472,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="36" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B36" s="20">
         <v>26</v>
       </c>
@@ -3477,7 +3522,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B37" s="20">
         <v>27</v>
       </c>
@@ -3525,7 +3570,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B38" s="20">
         <v>28</v>
       </c>
@@ -3575,7 +3620,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B39" s="20">
         <v>29</v>
       </c>
@@ -3625,7 +3670,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B40" s="20">
         <v>30</v>
       </c>
@@ -3675,7 +3720,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B41" s="20">
         <v>31</v>
       </c>
@@ -3725,7 +3770,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B42" s="20">
         <v>32</v>
       </c>
@@ -3775,7 +3820,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="43" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B43" s="20">
         <v>33</v>
       </c>
@@ -3825,7 +3870,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="44" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B44" s="20">
         <v>34</v>
       </c>
@@ -3873,7 +3918,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="45" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B45" s="20">
         <v>35</v>
       </c>
@@ -3921,7 +3966,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="46" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B46" s="20">
         <v>36</v>
       </c>
@@ -3969,7 +4014,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="47" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B47" s="20">
         <v>37</v>
       </c>
@@ -4017,7 +4062,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="48" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B48" s="20">
         <v>38</v>
       </c>
@@ -4065,7 +4110,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B49" s="20">
         <v>39</v>
       </c>
@@ -4113,7 +4158,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B50" s="20">
         <v>40</v>
       </c>
@@ -4161,7 +4206,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="51" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B51" s="20">
         <v>41</v>
       </c>
@@ -4209,7 +4254,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="52" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B52" s="20">
         <v>42</v>
       </c>
@@ -4237,7 +4282,7 @@
       </c>
       <c r="P52" s="22"/>
     </row>
-    <row r="53" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B53" s="20">
         <v>43</v>
       </c>
@@ -4268,7 +4313,7 @@
       </c>
       <c r="P53" s="22"/>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B54" s="20">
         <v>44</v>
       </c>
@@ -4299,7 +4344,7 @@
       </c>
       <c r="P54" s="22"/>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B55" s="20">
         <v>45</v>
       </c>
@@ -4330,7 +4375,7 @@
       </c>
       <c r="P55" s="22"/>
     </row>
-    <row r="56" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B56" s="20">
         <v>46</v>
       </c>
@@ -4361,7 +4406,7 @@
       </c>
       <c r="P56" s="22"/>
     </row>
-    <row r="57" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B57" s="20">
         <v>47</v>
       </c>
@@ -4392,7 +4437,7 @@
       </c>
       <c r="P57" s="22"/>
     </row>
-    <row r="58" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B58" s="20">
         <v>48</v>
       </c>
@@ -4423,7 +4468,7 @@
       </c>
       <c r="P58" s="22"/>
     </row>
-    <row r="59" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B59" s="20">
         <v>49</v>
       </c>
@@ -4454,7 +4499,7 @@
       </c>
       <c r="P59" s="22"/>
     </row>
-    <row r="60" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B60" s="20">
         <v>50</v>
       </c>
@@ -4485,7 +4530,7 @@
       </c>
       <c r="P60" s="22"/>
     </row>
-    <row r="61" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B61" s="20">
         <v>51</v>
       </c>
@@ -4516,7 +4561,7 @@
       </c>
       <c r="P61" s="22"/>
     </row>
-    <row r="62" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B62" s="20">
         <v>52</v>
       </c>
@@ -4547,7 +4592,7 @@
       </c>
       <c r="P62" s="22"/>
     </row>
-    <row r="63" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B63" s="20">
         <v>53</v>
       </c>
@@ -4578,7 +4623,7 @@
       </c>
       <c r="P63" s="22"/>
     </row>
-    <row r="64" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B64" s="20">
         <v>54</v>
       </c>
@@ -4609,7 +4654,7 @@
       </c>
       <c r="P64" s="22"/>
     </row>
-    <row r="65" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B65" s="20">
         <v>55</v>
       </c>
@@ -4640,7 +4685,7 @@
       </c>
       <c r="P65" s="22"/>
     </row>
-    <row r="66" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B66" s="20">
         <v>56</v>
       </c>
@@ -4671,7 +4716,7 @@
       </c>
       <c r="P66" s="22"/>
     </row>
-    <row r="67" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B67" s="20">
         <v>57</v>
       </c>
@@ -4702,7 +4747,7 @@
       </c>
       <c r="P67" s="22"/>
     </row>
-    <row r="68" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B68" s="20">
         <v>58</v>
       </c>
@@ -4733,7 +4778,7 @@
       </c>
       <c r="P68" s="22"/>
     </row>
-    <row r="69" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B69" s="20">
         <v>59</v>
       </c>
@@ -4764,7 +4809,7 @@
       </c>
       <c r="P69" s="22"/>
     </row>
-    <row r="70" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B70" s="20">
         <v>60</v>
       </c>
@@ -4795,7 +4840,7 @@
       </c>
       <c r="P70" s="22"/>
     </row>
-    <row r="71" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B71" s="20">
         <v>61</v>
       </c>
@@ -4826,7 +4871,7 @@
       </c>
       <c r="P71" s="22"/>
     </row>
-    <row r="72" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B72" s="20">
         <v>62</v>
       </c>
@@ -4857,7 +4902,7 @@
       </c>
       <c r="P72" s="22"/>
     </row>
-    <row r="73" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B73" s="20">
         <v>63</v>
       </c>
@@ -4888,7 +4933,7 @@
       </c>
       <c r="P73" s="22"/>
     </row>
-    <row r="74" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B74" s="20">
         <v>64</v>
       </c>
@@ -4919,7 +4964,7 @@
       </c>
       <c r="P74" s="22"/>
     </row>
-    <row r="75" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B75" s="20">
         <v>65</v>
       </c>
@@ -4950,7 +4995,7 @@
       </c>
       <c r="P75" s="22"/>
     </row>
-    <row r="76" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B76" s="20">
         <v>66</v>
       </c>
@@ -4981,7 +5026,7 @@
       </c>
       <c r="P76" s="22"/>
     </row>
-    <row r="77" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B77" s="20">
         <v>67</v>
       </c>
@@ -5012,7 +5057,7 @@
       </c>
       <c r="P77" s="22"/>
     </row>
-    <row r="78" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B78" s="20">
         <v>68</v>
       </c>
@@ -5043,7 +5088,7 @@
       </c>
       <c r="P78" s="22"/>
     </row>
-    <row r="79" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B79" s="20">
         <v>69</v>
       </c>
@@ -5074,7 +5119,7 @@
       </c>
       <c r="P79" s="22"/>
     </row>
-    <row r="80" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B80" s="20">
         <v>70</v>
       </c>
@@ -5105,7 +5150,7 @@
       </c>
       <c r="P80" s="22"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B81" s="20">
         <v>71</v>
       </c>
@@ -5136,7 +5181,7 @@
       </c>
       <c r="P81" s="22"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B82" s="20">
         <v>72</v>
       </c>
@@ -5167,7 +5212,7 @@
       </c>
       <c r="P82" s="22"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B83" s="20">
         <v>73</v>
       </c>
@@ -5198,7 +5243,7 @@
       </c>
       <c r="P83" s="22"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B84" s="20">
         <v>74</v>
       </c>
@@ -5229,7 +5274,7 @@
       </c>
       <c r="P84" s="22"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B85" s="20">
         <v>75</v>
       </c>
@@ -5260,7 +5305,7 @@
       </c>
       <c r="P85" s="22"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B86" s="20">
         <v>76</v>
       </c>
@@ -5291,7 +5336,7 @@
       </c>
       <c r="P86" s="22"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B87" s="20">
         <v>77</v>
       </c>
@@ -5322,7 +5367,7 @@
       </c>
       <c r="P87" s="22"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B88" s="20">
         <v>78</v>
       </c>
@@ -5353,7 +5398,7 @@
       </c>
       <c r="P88" s="22"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B89" s="20">
         <v>79</v>
       </c>
@@ -5384,7 +5429,7 @@
       </c>
       <c r="P89" s="22"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B90" s="20">
         <v>80</v>
       </c>
@@ -5415,7 +5460,7 @@
       </c>
       <c r="P90" s="22"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B91" s="20">
         <v>81</v>
       </c>
@@ -5446,7 +5491,7 @@
       </c>
       <c r="P91" s="22"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B92" s="20">
         <v>82</v>
       </c>
@@ -5477,7 +5522,7 @@
       </c>
       <c r="P92" s="22"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B93" s="20">
         <v>83</v>
       </c>
@@ -5508,7 +5553,7 @@
       </c>
       <c r="P93" s="22"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B94" s="20">
         <v>84</v>
       </c>
@@ -5539,7 +5584,7 @@
       </c>
       <c r="P94" s="22"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B95" s="20">
         <v>85</v>
       </c>
@@ -5570,7 +5615,7 @@
       </c>
       <c r="P95" s="22"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B96" s="20">
         <v>86</v>
       </c>
@@ -5601,7 +5646,7 @@
       </c>
       <c r="P96" s="22"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B97" s="20">
         <v>87</v>
       </c>
@@ -5632,7 +5677,7 @@
       </c>
       <c r="P97" s="22"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B98" s="20">
         <v>88</v>
       </c>
@@ -5663,7 +5708,7 @@
       </c>
       <c r="P98" s="22"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B99" s="20">
         <v>89</v>
       </c>
@@ -5694,7 +5739,7 @@
       </c>
       <c r="P99" s="22"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B100" s="20">
         <v>90</v>
       </c>
@@ -5725,7 +5770,7 @@
       </c>
       <c r="P100" s="22"/>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B101" s="20">
         <v>91</v>
       </c>
@@ -5756,7 +5801,7 @@
       </c>
       <c r="P101" s="22"/>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B102" s="20">
         <v>92</v>
       </c>
@@ -5787,7 +5832,7 @@
       </c>
       <c r="P102" s="22"/>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B103" s="20">
         <v>93</v>
       </c>
@@ -5818,7 +5863,7 @@
       </c>
       <c r="P103" s="22"/>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B104" s="20">
         <v>94</v>
       </c>
@@ -5849,7 +5894,7 @@
       </c>
       <c r="P104" s="22"/>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B105" s="20">
         <v>95</v>
       </c>
@@ -5880,7 +5925,7 @@
       </c>
       <c r="P105" s="22"/>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B106" s="20">
         <v>96</v>
       </c>
@@ -5911,7 +5956,7 @@
       </c>
       <c r="P106" s="22"/>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B107" s="20">
         <v>97</v>
       </c>
@@ -5942,7 +5987,7 @@
       </c>
       <c r="P107" s="22"/>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B108" s="20">
         <v>98</v>
       </c>
@@ -5973,7 +6018,7 @@
       </c>
       <c r="P108" s="22"/>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B109" s="20">
         <v>99</v>
       </c>
@@ -6004,7 +6049,7 @@
       </c>
       <c r="P109" s="22"/>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B110" s="20">
         <v>100</v>
       </c>
@@ -6143,13 +6188,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:P110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="15" width="18.88671875" customWidth="1"/>
-    <col min="16" max="16" width="64.5546875" customWidth="1"/>
+    <col min="3" max="15" width="18.90625" customWidth="1"/>
+    <col min="16" max="16" width="64.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C2" s="63" t="s">
         <v>71</v>
       </c>
@@ -6167,7 +6212,7 @@
       <c r="O2" s="63"/>
       <c r="P2" s="63"/>
     </row>
-    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C4" s="64" t="s">
         <v>10</v>
       </c>
@@ -6185,7 +6230,7 @@
       <c r="O4" s="64"/>
       <c r="P4" s="64"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -6201,7 +6246,7 @@
       <c r="O5" s="9"/>
       <c r="P5" s="9"/>
     </row>
-    <row r="6" spans="2:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C6" s="65" t="s">
         <v>11</v>
       </c>
@@ -6224,7 +6269,7 @@
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C7" s="65"/>
       <c r="D7" s="12" t="s">
         <v>13</v>
@@ -6235,7 +6280,7 @@
       </c>
       <c r="J7" s="14"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B9" s="15"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
@@ -6258,7 +6303,7 @@
       <c r="O9" s="66"/>
       <c r="P9" s="16"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>17</v>
       </c>
@@ -6305,7 +6350,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B11" s="20">
         <v>1</v>
       </c>
@@ -6354,7 +6399,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B12" s="20">
         <v>2</v>
       </c>
@@ -6403,7 +6448,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B13" s="20">
         <v>3</v>
       </c>
@@ -6454,7 +6499,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B14" s="20">
         <v>4</v>
       </c>
@@ -6505,7 +6550,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B15" s="20">
         <v>5</v>
       </c>
@@ -6556,7 +6601,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B16" s="20">
         <v>6</v>
       </c>
@@ -6607,7 +6652,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B17" s="20">
         <v>7</v>
       </c>
@@ -6656,7 +6701,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B18" s="20">
         <v>8</v>
       </c>
@@ -6705,7 +6750,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B19" s="20">
         <v>9</v>
       </c>
@@ -6754,7 +6799,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B20" s="20">
         <v>10</v>
       </c>
@@ -6803,7 +6848,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B21" s="20">
         <v>11</v>
       </c>
@@ -6852,7 +6897,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B22" s="20">
         <v>12</v>
       </c>
@@ -6901,7 +6946,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B23" s="20">
         <v>13</v>
       </c>
@@ -6950,7 +6995,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B24" s="20">
         <v>14</v>
       </c>
@@ -6999,7 +7044,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B25" s="20">
         <v>15</v>
       </c>
@@ -7048,7 +7093,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B26" s="20">
         <v>16</v>
       </c>
@@ -7079,7 +7124,7 @@
       </c>
       <c r="P26" s="22"/>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B27" s="20">
         <v>17</v>
       </c>
@@ -7110,7 +7155,7 @@
       </c>
       <c r="P27" s="22"/>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B28" s="20">
         <v>18</v>
       </c>
@@ -7141,7 +7186,7 @@
       </c>
       <c r="P28" s="22"/>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="20">
         <v>19</v>
       </c>
@@ -7172,7 +7217,7 @@
       </c>
       <c r="P29" s="22"/>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B30" s="20">
         <v>20</v>
       </c>
@@ -7203,7 +7248,7 @@
       </c>
       <c r="P30" s="22"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B31" s="20">
         <v>21</v>
       </c>
@@ -7234,7 +7279,7 @@
       </c>
       <c r="P31" s="22"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B32" s="20">
         <v>22</v>
       </c>
@@ -7265,7 +7310,7 @@
       </c>
       <c r="P32" s="22"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B33" s="20">
         <v>23</v>
       </c>
@@ -7296,7 +7341,7 @@
       </c>
       <c r="P33" s="22"/>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B34" s="20">
         <v>24</v>
       </c>
@@ -7327,7 +7372,7 @@
       </c>
       <c r="P34" s="22"/>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B35" s="20">
         <v>25</v>
       </c>
@@ -7358,7 +7403,7 @@
       </c>
       <c r="P35" s="22"/>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B36" s="20">
         <v>26</v>
       </c>
@@ -7389,7 +7434,7 @@
       </c>
       <c r="P36" s="22"/>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B37" s="20">
         <v>27</v>
       </c>
@@ -7420,7 +7465,7 @@
       </c>
       <c r="P37" s="22"/>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B38" s="20">
         <v>28</v>
       </c>
@@ -7451,7 +7496,7 @@
       </c>
       <c r="P38" s="22"/>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B39" s="20">
         <v>29</v>
       </c>
@@ -7482,7 +7527,7 @@
       </c>
       <c r="P39" s="22"/>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B40" s="20">
         <v>30</v>
       </c>
@@ -7513,7 +7558,7 @@
       </c>
       <c r="P40" s="22"/>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B41" s="20">
         <v>31</v>
       </c>
@@ -7544,7 +7589,7 @@
       </c>
       <c r="P41" s="22"/>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B42" s="20">
         <v>32</v>
       </c>
@@ -7575,7 +7620,7 @@
       </c>
       <c r="P42" s="22"/>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B43" s="20">
         <v>33</v>
       </c>
@@ -7606,7 +7651,7 @@
       </c>
       <c r="P43" s="22"/>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B44" s="20">
         <v>34</v>
       </c>
@@ -7637,7 +7682,7 @@
       </c>
       <c r="P44" s="22"/>
     </row>
-    <row r="45" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B45" s="20">
         <v>35</v>
       </c>
@@ -7668,7 +7713,7 @@
       </c>
       <c r="P45" s="22"/>
     </row>
-    <row r="46" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B46" s="20">
         <v>36</v>
       </c>
@@ -7699,7 +7744,7 @@
       </c>
       <c r="P46" s="22"/>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B47" s="20">
         <v>37</v>
       </c>
@@ -7730,7 +7775,7 @@
       </c>
       <c r="P47" s="22"/>
     </row>
-    <row r="48" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B48" s="20">
         <v>38</v>
       </c>
@@ -7761,7 +7806,7 @@
       </c>
       <c r="P48" s="22"/>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B49" s="20">
         <v>39</v>
       </c>
@@ -7792,7 +7837,7 @@
       </c>
       <c r="P49" s="22"/>
     </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B50" s="20">
         <v>40</v>
       </c>
@@ -7823,7 +7868,7 @@
       </c>
       <c r="P50" s="22"/>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B51" s="20">
         <v>41</v>
       </c>
@@ -7854,7 +7899,7 @@
       </c>
       <c r="P51" s="22"/>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B52" s="20">
         <v>42</v>
       </c>
@@ -7885,7 +7930,7 @@
       </c>
       <c r="P52" s="22"/>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B53" s="20">
         <v>43</v>
       </c>
@@ -7916,7 +7961,7 @@
       </c>
       <c r="P53" s="22"/>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B54" s="20">
         <v>44</v>
       </c>
@@ -7947,7 +7992,7 @@
       </c>
       <c r="P54" s="22"/>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B55" s="20">
         <v>45</v>
       </c>
@@ -7978,7 +8023,7 @@
       </c>
       <c r="P55" s="22"/>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B56" s="20">
         <v>46</v>
       </c>
@@ -8009,7 +8054,7 @@
       </c>
       <c r="P56" s="22"/>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B57" s="20">
         <v>47</v>
       </c>
@@ -8040,7 +8085,7 @@
       </c>
       <c r="P57" s="22"/>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B58" s="20">
         <v>48</v>
       </c>
@@ -8071,7 +8116,7 @@
       </c>
       <c r="P58" s="22"/>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B59" s="20">
         <v>49</v>
       </c>
@@ -8102,7 +8147,7 @@
       </c>
       <c r="P59" s="22"/>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B60" s="20">
         <v>50</v>
       </c>
@@ -8133,7 +8178,7 @@
       </c>
       <c r="P60" s="22"/>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B61" s="20">
         <v>51</v>
       </c>
@@ -8164,7 +8209,7 @@
       </c>
       <c r="P61" s="22"/>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B62" s="20">
         <v>52</v>
       </c>
@@ -8195,7 +8240,7 @@
       </c>
       <c r="P62" s="22"/>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B63" s="20">
         <v>53</v>
       </c>
@@ -8226,7 +8271,7 @@
       </c>
       <c r="P63" s="22"/>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B64" s="20">
         <v>54</v>
       </c>
@@ -8257,7 +8302,7 @@
       </c>
       <c r="P64" s="22"/>
     </row>
-    <row r="65" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B65" s="20">
         <v>55</v>
       </c>
@@ -8288,7 +8333,7 @@
       </c>
       <c r="P65" s="22"/>
     </row>
-    <row r="66" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B66" s="20">
         <v>56</v>
       </c>
@@ -8319,7 +8364,7 @@
       </c>
       <c r="P66" s="22"/>
     </row>
-    <row r="67" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B67" s="20">
         <v>57</v>
       </c>
@@ -8350,7 +8395,7 @@
       </c>
       <c r="P67" s="22"/>
     </row>
-    <row r="68" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B68" s="20">
         <v>58</v>
       </c>
@@ -8381,7 +8426,7 @@
       </c>
       <c r="P68" s="22"/>
     </row>
-    <row r="69" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B69" s="20">
         <v>59</v>
       </c>
@@ -8412,7 +8457,7 @@
       </c>
       <c r="P69" s="22"/>
     </row>
-    <row r="70" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B70" s="20">
         <v>60</v>
       </c>
@@ -8443,7 +8488,7 @@
       </c>
       <c r="P70" s="22"/>
     </row>
-    <row r="71" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B71" s="20">
         <v>61</v>
       </c>
@@ -8474,7 +8519,7 @@
       </c>
       <c r="P71" s="22"/>
     </row>
-    <row r="72" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B72" s="20">
         <v>62</v>
       </c>
@@ -8505,7 +8550,7 @@
       </c>
       <c r="P72" s="22"/>
     </row>
-    <row r="73" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B73" s="20">
         <v>63</v>
       </c>
@@ -8536,7 +8581,7 @@
       </c>
       <c r="P73" s="22"/>
     </row>
-    <row r="74" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B74" s="20">
         <v>64</v>
       </c>
@@ -8567,7 +8612,7 @@
       </c>
       <c r="P74" s="22"/>
     </row>
-    <row r="75" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B75" s="20">
         <v>65</v>
       </c>
@@ -8598,7 +8643,7 @@
       </c>
       <c r="P75" s="22"/>
     </row>
-    <row r="76" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B76" s="20">
         <v>66</v>
       </c>
@@ -8629,7 +8674,7 @@
       </c>
       <c r="P76" s="22"/>
     </row>
-    <row r="77" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B77" s="20">
         <v>67</v>
       </c>
@@ -8660,7 +8705,7 @@
       </c>
       <c r="P77" s="22"/>
     </row>
-    <row r="78" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B78" s="20">
         <v>68</v>
       </c>
@@ -8691,7 +8736,7 @@
       </c>
       <c r="P78" s="22"/>
     </row>
-    <row r="79" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B79" s="20">
         <v>69</v>
       </c>
@@ -8722,7 +8767,7 @@
       </c>
       <c r="P79" s="22"/>
     </row>
-    <row r="80" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B80" s="20">
         <v>70</v>
       </c>
@@ -8753,7 +8798,7 @@
       </c>
       <c r="P80" s="22"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B81" s="20">
         <v>71</v>
       </c>
@@ -8784,7 +8829,7 @@
       </c>
       <c r="P81" s="22"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B82" s="20">
         <v>72</v>
       </c>
@@ -8815,7 +8860,7 @@
       </c>
       <c r="P82" s="22"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B83" s="20">
         <v>73</v>
       </c>
@@ -8846,7 +8891,7 @@
       </c>
       <c r="P83" s="22"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B84" s="20">
         <v>74</v>
       </c>
@@ -8877,7 +8922,7 @@
       </c>
       <c r="P84" s="22"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B85" s="20">
         <v>75</v>
       </c>
@@ -8908,7 +8953,7 @@
       </c>
       <c r="P85" s="22"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B86" s="20">
         <v>76</v>
       </c>
@@ -8939,7 +8984,7 @@
       </c>
       <c r="P86" s="22"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B87" s="20">
         <v>77</v>
       </c>
@@ -8970,7 +9015,7 @@
       </c>
       <c r="P87" s="22"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B88" s="20">
         <v>78</v>
       </c>
@@ -9001,7 +9046,7 @@
       </c>
       <c r="P88" s="22"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B89" s="20">
         <v>79</v>
       </c>
@@ -9032,7 +9077,7 @@
       </c>
       <c r="P89" s="22"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B90" s="20">
         <v>80</v>
       </c>
@@ -9063,7 +9108,7 @@
       </c>
       <c r="P90" s="22"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B91" s="20">
         <v>81</v>
       </c>
@@ -9094,7 +9139,7 @@
       </c>
       <c r="P91" s="22"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B92" s="20">
         <v>82</v>
       </c>
@@ -9125,7 +9170,7 @@
       </c>
       <c r="P92" s="22"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B93" s="20">
         <v>83</v>
       </c>
@@ -9156,7 +9201,7 @@
       </c>
       <c r="P93" s="22"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B94" s="20">
         <v>84</v>
       </c>
@@ -9187,7 +9232,7 @@
       </c>
       <c r="P94" s="22"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B95" s="20">
         <v>85</v>
       </c>
@@ -9218,7 +9263,7 @@
       </c>
       <c r="P95" s="22"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B96" s="20">
         <v>86</v>
       </c>
@@ -9249,7 +9294,7 @@
       </c>
       <c r="P96" s="22"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B97" s="20">
         <v>87</v>
       </c>
@@ -9280,7 +9325,7 @@
       </c>
       <c r="P97" s="22"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B98" s="20">
         <v>88</v>
       </c>
@@ -9311,7 +9356,7 @@
       </c>
       <c r="P98" s="22"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B99" s="20">
         <v>89</v>
       </c>
@@ -9342,7 +9387,7 @@
       </c>
       <c r="P99" s="22"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B100" s="20">
         <v>90</v>
       </c>
@@ -9373,7 +9418,7 @@
       </c>
       <c r="P100" s="22"/>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B101" s="20">
         <v>91</v>
       </c>
@@ -9404,7 +9449,7 @@
       </c>
       <c r="P101" s="22"/>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B102" s="20">
         <v>92</v>
       </c>
@@ -9435,7 +9480,7 @@
       </c>
       <c r="P102" s="22"/>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B103" s="20">
         <v>93</v>
       </c>
@@ -9466,7 +9511,7 @@
       </c>
       <c r="P103" s="22"/>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B104" s="20">
         <v>94</v>
       </c>
@@ -9497,7 +9542,7 @@
       </c>
       <c r="P104" s="22"/>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B105" s="20">
         <v>95</v>
       </c>
@@ -9528,7 +9573,7 @@
       </c>
       <c r="P105" s="22"/>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B106" s="20">
         <v>96</v>
       </c>
@@ -9559,7 +9604,7 @@
       </c>
       <c r="P106" s="22"/>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B107" s="20">
         <v>97</v>
       </c>
@@ -9590,7 +9635,7 @@
       </c>
       <c r="P107" s="22"/>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B108" s="20">
         <v>98</v>
       </c>
@@ -9621,7 +9666,7 @@
       </c>
       <c r="P108" s="22"/>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B109" s="20">
         <v>99</v>
       </c>
@@ -9652,7 +9697,7 @@
       </c>
       <c r="P109" s="22"/>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B110" s="20">
         <v>100</v>
       </c>
@@ -9789,14 +9834,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="B2:P110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:P110"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="15" width="18.88671875" customWidth="1"/>
-    <col min="16" max="16" width="64.5546875" customWidth="1"/>
+    <col min="3" max="15" width="18.90625" customWidth="1"/>
+    <col min="16" max="16" width="64.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C2" s="63" t="s">
         <v>87</v>
       </c>
@@ -9814,7 +9859,7 @@
       <c r="O2" s="63"/>
       <c r="P2" s="63"/>
     </row>
-    <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C4" s="64" t="s">
         <v>10</v>
       </c>
@@ -9832,7 +9877,7 @@
       <c r="O4" s="64"/>
       <c r="P4" s="64"/>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -9848,7 +9893,11 @@
       <c r="O5" s="9"/>
       <c r="P5" s="9"/>
     </row>
-    <row r="6" spans="2:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" cm="1">
+        <f t="array" aca="1" ref="B6" ca="1">B6:P15</f>
+        <v>0</v>
+      </c>
       <c r="C6" s="65" t="s">
         <v>11</v>
       </c>
@@ -9857,7 +9906,7 @@
       </c>
       <c r="E6" s="11">
         <f>SUM(N11:N110)</f>
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
@@ -9871,18 +9920,18 @@
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C7" s="65"/>
       <c r="D7" s="12" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="13">
         <f>SUM(O11:O110)</f>
-        <v>0</v>
+        <v>255</v>
       </c>
       <c r="J7" s="14"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B9" s="15"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
@@ -9905,7 +9954,7 @@
       <c r="O9" s="66"/>
       <c r="P9" s="16"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>17</v>
       </c>
@@ -9952,162 +10001,263 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B11" s="20">
         <v>1</v>
       </c>
       <c r="C11" s="21" t="str">
         <f>IF(ISBLANK(D11), "", _xlfn.CONCAT("T", TEXT(B11, "0000"), "/", VLOOKUP(D11, Internal!$B$35:C$39, 2, FALSE()), IF(OR(D11="QA", D11="Revision"), _xlfn.CONCAT("/", H11), "")))</f>
-        <v/>
-      </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="22"/>
+        <v>T0001/M</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>74</v>
+      </c>
       <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
+      <c r="I11" s="24">
+        <v>46158.375</v>
+      </c>
+      <c r="J11" s="24">
+        <v>46158.416666666664</v>
+      </c>
       <c r="K11" s="25" t="str">
         <f t="shared" ref="K11:K42" ca="1" si="0">IF(OR(I11="",J11=""),"",IF(AND(J11&lt;&gt;"",I11&gt;=NOW()),"Planned",IF(AND(J11&lt;&gt;"",J11&lt;NOW()),"Completed","Ongoing")))</f>
-        <v/>
-      </c>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="25" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L11" s="26">
+        <v>1</v>
+      </c>
+      <c r="M11" s="26">
+        <v>1</v>
+      </c>
+      <c r="N11" s="25">
         <f>IF(ISBLANK(L11), "", L11*VLOOKUP($F11,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="O11" s="25" t="str">
+        <v>40</v>
+      </c>
+      <c r="O11" s="25">
         <f>IF(ISBLANK(M11), "", M11*VLOOKUP($F11,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="P11" s="22"/>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="P11" s="22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B12" s="20">
         <v>2</v>
       </c>
       <c r="C12" s="21" t="str">
         <f>IF(ISBLANK(D12), "", _xlfn.CONCAT("T", TEXT(B12, "0000"), "/", VLOOKUP(D12, Internal!$B$35:C$39, 2, FALSE()), IF(OR(D12="QA", D12="Revision"), _xlfn.CONCAT("/", H12), "")))</f>
-        <v/>
-      </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
+        <v>T0002/M</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="I12" s="24">
+        <v>46158.416666666664</v>
+      </c>
+      <c r="J12" s="24">
+        <v>46158.458333333336</v>
+      </c>
       <c r="K12" s="25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L12" s="26"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="25" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L12" s="26">
+        <v>1</v>
+      </c>
+      <c r="M12" s="26">
+        <v>1</v>
+      </c>
+      <c r="N12" s="25">
         <f>IF(ISBLANK(L12), "", L12*VLOOKUP($F12,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="O12" s="25" t="str">
+        <v>40</v>
+      </c>
+      <c r="O12" s="25">
         <f>IF(ISBLANK(M12), "", M12*VLOOKUP($F12,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="P12" s="22"/>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="P12" s="22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B13" s="20">
         <v>3</v>
       </c>
       <c r="C13" s="21" t="str">
         <f>IF(ISBLANK(D13), "", _xlfn.CONCAT("T", TEXT(B13, "0000"), "/", VLOOKUP(D13, Internal!$B$35:C$39, 2, FALSE()), IF(OR(D13="QA", D13="Revision"), _xlfn.CONCAT("/", H13), "")))</f>
-        <v/>
-      </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
+        <v>T0003/D</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="I13" s="24">
+        <v>46158.458333333336</v>
+      </c>
+      <c r="J13" s="24">
+        <v>46158.666666666664</v>
+      </c>
       <c r="K13" s="25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L13" s="26"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="25" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L13" s="26">
+        <v>4</v>
+      </c>
+      <c r="M13" s="26">
+        <v>5</v>
+      </c>
+      <c r="N13" s="25">
         <f>IF(ISBLANK(L13), "", L13*VLOOKUP($F13,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="O13" s="25" t="str">
+        <v>100</v>
+      </c>
+      <c r="O13" s="25">
         <f>IF(ISBLANK(M13), "", M13*VLOOKUP($F13,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="P13" s="22"/>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+      <c r="P13" s="22" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B14" s="20">
         <v>4</v>
       </c>
       <c r="C14" s="21" t="str">
         <f>IF(ISBLANK(D14), "", _xlfn.CONCAT("T", TEXT(B14, "0000"), "/", VLOOKUP(D14, Internal!$B$35:C$39, 2, FALSE()), IF(OR(D14="QA", D14="Revision"), _xlfn.CONCAT("/", H14), "")))</f>
-        <v/>
-      </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
+        <v>T0004/QA/T0003/D</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="I14" s="24">
+        <v>46158.708333333336</v>
+      </c>
+      <c r="J14" s="24">
+        <v>46158.791666666664</v>
+      </c>
       <c r="K14" s="25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L14" s="26"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="25" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L14" s="26">
+        <v>2</v>
+      </c>
+      <c r="M14" s="26">
+        <v>2</v>
+      </c>
+      <c r="N14" s="25">
         <f>IF(ISBLANK(L14), "", L14*VLOOKUP($F14,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="O14" s="25" t="str">
+        <v>50</v>
+      </c>
+      <c r="O14" s="25">
         <f>IF(ISBLANK(M14), "", M14*VLOOKUP($F14,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="P14" s="22"/>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+      <c r="P14" s="22" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>168</v>
+      </c>
       <c r="B15" s="20">
         <v>5</v>
       </c>
       <c r="C15" s="21" t="str">
         <f>IF(ISBLANK(D15), "", _xlfn.CONCAT("T", TEXT(B15, "0000"), "/", VLOOKUP(D15, Internal!$B$35:C$39, 2, FALSE()), IF(OR(D15="QA", D15="Revision"), _xlfn.CONCAT("/", H15), "")))</f>
-        <v/>
-      </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
+        <v>T0005/R/T0003/D</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="I15" s="24">
+        <v>46160.354166666664</v>
+      </c>
+      <c r="J15" s="24">
+        <v>46160.395833333336</v>
+      </c>
       <c r="K15" s="25" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="L15" s="26"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="25" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="L15" s="26">
+        <v>1</v>
+      </c>
+      <c r="M15" s="26">
+        <v>1</v>
+      </c>
+      <c r="N15" s="25">
         <f>IF(ISBLANK(L15), "", L15*VLOOKUP($F15,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="O15" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="O15" s="25">
         <f>IF(ISBLANK(M15), "", M15*VLOOKUP($F15,Internal!$B$26:$C$32,2,FALSE()))</f>
-        <v/>
-      </c>
-      <c r="P15" s="22"/>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="P15" s="22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B16" s="20">
         <v>6</v>
       </c>
@@ -10138,7 +10288,7 @@
       </c>
       <c r="P16" s="22"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B17" s="20">
         <v>7</v>
       </c>
@@ -10169,7 +10319,7 @@
       </c>
       <c r="P17" s="22"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B18" s="20">
         <v>8</v>
       </c>
@@ -10200,7 +10350,7 @@
       </c>
       <c r="P18" s="22"/>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B19" s="20">
         <v>9</v>
       </c>
@@ -10231,7 +10381,7 @@
       </c>
       <c r="P19" s="22"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B20" s="20">
         <v>10</v>
       </c>
@@ -10262,7 +10412,7 @@
       </c>
       <c r="P20" s="22"/>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B21" s="20">
         <v>11</v>
       </c>
@@ -10293,7 +10443,7 @@
       </c>
       <c r="P21" s="22"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B22" s="20">
         <v>12</v>
       </c>
@@ -10324,7 +10474,7 @@
       </c>
       <c r="P22" s="22"/>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B23" s="20">
         <v>13</v>
       </c>
@@ -10355,7 +10505,7 @@
       </c>
       <c r="P23" s="22"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B24" s="20">
         <v>14</v>
       </c>
@@ -10386,7 +10536,7 @@
       </c>
       <c r="P24" s="22"/>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B25" s="20">
         <v>15</v>
       </c>
@@ -10417,7 +10567,7 @@
       </c>
       <c r="P25" s="22"/>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B26" s="20">
         <v>16</v>
       </c>
@@ -10448,7 +10598,7 @@
       </c>
       <c r="P26" s="22"/>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B27" s="20">
         <v>17</v>
       </c>
@@ -10479,7 +10629,7 @@
       </c>
       <c r="P27" s="22"/>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B28" s="20">
         <v>18</v>
       </c>
@@ -10510,7 +10660,7 @@
       </c>
       <c r="P28" s="22"/>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="20">
         <v>19</v>
       </c>
@@ -10541,7 +10691,7 @@
       </c>
       <c r="P29" s="22"/>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B30" s="20">
         <v>20</v>
       </c>
@@ -10572,7 +10722,7 @@
       </c>
       <c r="P30" s="22"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B31" s="20">
         <v>21</v>
       </c>
@@ -10603,7 +10753,7 @@
       </c>
       <c r="P31" s="22"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B32" s="20">
         <v>22</v>
       </c>
@@ -10634,7 +10784,7 @@
       </c>
       <c r="P32" s="22"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B33" s="20">
         <v>23</v>
       </c>
@@ -10665,7 +10815,7 @@
       </c>
       <c r="P33" s="22"/>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B34" s="20">
         <v>24</v>
       </c>
@@ -10696,7 +10846,7 @@
       </c>
       <c r="P34" s="22"/>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B35" s="20">
         <v>25</v>
       </c>
@@ -10727,7 +10877,7 @@
       </c>
       <c r="P35" s="22"/>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B36" s="20">
         <v>26</v>
       </c>
@@ -10758,7 +10908,7 @@
       </c>
       <c r="P36" s="22"/>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B37" s="20">
         <v>27</v>
       </c>
@@ -10789,7 +10939,7 @@
       </c>
       <c r="P37" s="22"/>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B38" s="20">
         <v>28</v>
       </c>
@@ -10820,7 +10970,7 @@
       </c>
       <c r="P38" s="22"/>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B39" s="20">
         <v>29</v>
       </c>
@@ -10851,7 +11001,7 @@
       </c>
       <c r="P39" s="22"/>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B40" s="20">
         <v>30</v>
       </c>
@@ -10882,7 +11032,7 @@
       </c>
       <c r="P40" s="22"/>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B41" s="20">
         <v>31</v>
       </c>
@@ -10913,7 +11063,7 @@
       </c>
       <c r="P41" s="22"/>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B42" s="20">
         <v>32</v>
       </c>
@@ -10944,7 +11094,7 @@
       </c>
       <c r="P42" s="22"/>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B43" s="20">
         <v>33</v>
       </c>
@@ -10975,7 +11125,7 @@
       </c>
       <c r="P43" s="22"/>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B44" s="20">
         <v>34</v>
       </c>
@@ -11006,7 +11156,7 @@
       </c>
       <c r="P44" s="22"/>
     </row>
-    <row r="45" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B45" s="20">
         <v>35</v>
       </c>
@@ -11037,7 +11187,7 @@
       </c>
       <c r="P45" s="22"/>
     </row>
-    <row r="46" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B46" s="20">
         <v>36</v>
       </c>
@@ -11068,7 +11218,7 @@
       </c>
       <c r="P46" s="22"/>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B47" s="20">
         <v>37</v>
       </c>
@@ -11099,7 +11249,7 @@
       </c>
       <c r="P47" s="22"/>
     </row>
-    <row r="48" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B48" s="20">
         <v>38</v>
       </c>
@@ -11130,7 +11280,7 @@
       </c>
       <c r="P48" s="22"/>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B49" s="20">
         <v>39</v>
       </c>
@@ -11161,7 +11311,7 @@
       </c>
       <c r="P49" s="22"/>
     </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B50" s="20">
         <v>40</v>
       </c>
@@ -11192,7 +11342,7 @@
       </c>
       <c r="P50" s="22"/>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B51" s="20">
         <v>41</v>
       </c>
@@ -11223,7 +11373,7 @@
       </c>
       <c r="P51" s="22"/>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B52" s="20">
         <v>42</v>
       </c>
@@ -11254,7 +11404,7 @@
       </c>
       <c r="P52" s="22"/>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B53" s="20">
         <v>43</v>
       </c>
@@ -11285,7 +11435,7 @@
       </c>
       <c r="P53" s="22"/>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B54" s="20">
         <v>44</v>
       </c>
@@ -11316,7 +11466,7 @@
       </c>
       <c r="P54" s="22"/>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B55" s="20">
         <v>45</v>
       </c>
@@ -11347,7 +11497,7 @@
       </c>
       <c r="P55" s="22"/>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B56" s="20">
         <v>46</v>
       </c>
@@ -11378,7 +11528,7 @@
       </c>
       <c r="P56" s="22"/>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B57" s="20">
         <v>47</v>
       </c>
@@ -11409,7 +11559,7 @@
       </c>
       <c r="P57" s="22"/>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B58" s="20">
         <v>48</v>
       </c>
@@ -11440,7 +11590,7 @@
       </c>
       <c r="P58" s="22"/>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B59" s="20">
         <v>49</v>
       </c>
@@ -11471,7 +11621,7 @@
       </c>
       <c r="P59" s="22"/>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B60" s="20">
         <v>50</v>
       </c>
@@ -11502,7 +11652,7 @@
       </c>
       <c r="P60" s="22"/>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B61" s="20">
         <v>51</v>
       </c>
@@ -11533,7 +11683,7 @@
       </c>
       <c r="P61" s="22"/>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B62" s="20">
         <v>52</v>
       </c>
@@ -11564,7 +11714,7 @@
       </c>
       <c r="P62" s="22"/>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B63" s="20">
         <v>53</v>
       </c>
@@ -11595,7 +11745,7 @@
       </c>
       <c r="P63" s="22"/>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B64" s="20">
         <v>54</v>
       </c>
@@ -11626,7 +11776,7 @@
       </c>
       <c r="P64" s="22"/>
     </row>
-    <row r="65" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B65" s="20">
         <v>55</v>
       </c>
@@ -11657,7 +11807,7 @@
       </c>
       <c r="P65" s="22"/>
     </row>
-    <row r="66" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B66" s="20">
         <v>56</v>
       </c>
@@ -11688,7 +11838,7 @@
       </c>
       <c r="P66" s="22"/>
     </row>
-    <row r="67" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B67" s="20">
         <v>57</v>
       </c>
@@ -11719,7 +11869,7 @@
       </c>
       <c r="P67" s="22"/>
     </row>
-    <row r="68" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B68" s="20">
         <v>58</v>
       </c>
@@ -11750,7 +11900,7 @@
       </c>
       <c r="P68" s="22"/>
     </row>
-    <row r="69" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B69" s="20">
         <v>59</v>
       </c>
@@ -11781,7 +11931,7 @@
       </c>
       <c r="P69" s="22"/>
     </row>
-    <row r="70" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B70" s="20">
         <v>60</v>
       </c>
@@ -11812,7 +11962,7 @@
       </c>
       <c r="P70" s="22"/>
     </row>
-    <row r="71" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B71" s="20">
         <v>61</v>
       </c>
@@ -11843,7 +11993,7 @@
       </c>
       <c r="P71" s="22"/>
     </row>
-    <row r="72" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B72" s="20">
         <v>62</v>
       </c>
@@ -11874,7 +12024,7 @@
       </c>
       <c r="P72" s="22"/>
     </row>
-    <row r="73" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B73" s="20">
         <v>63</v>
       </c>
@@ -11905,7 +12055,7 @@
       </c>
       <c r="P73" s="22"/>
     </row>
-    <row r="74" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B74" s="20">
         <v>64</v>
       </c>
@@ -11936,7 +12086,7 @@
       </c>
       <c r="P74" s="22"/>
     </row>
-    <row r="75" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B75" s="20">
         <v>65</v>
       </c>
@@ -11967,7 +12117,7 @@
       </c>
       <c r="P75" s="22"/>
     </row>
-    <row r="76" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B76" s="20">
         <v>66</v>
       </c>
@@ -11998,7 +12148,7 @@
       </c>
       <c r="P76" s="22"/>
     </row>
-    <row r="77" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B77" s="20">
         <v>67</v>
       </c>
@@ -12029,7 +12179,7 @@
       </c>
       <c r="P77" s="22"/>
     </row>
-    <row r="78" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B78" s="20">
         <v>68</v>
       </c>
@@ -12060,7 +12210,7 @@
       </c>
       <c r="P78" s="22"/>
     </row>
-    <row r="79" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B79" s="20">
         <v>69</v>
       </c>
@@ -12091,7 +12241,7 @@
       </c>
       <c r="P79" s="22"/>
     </row>
-    <row r="80" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B80" s="20">
         <v>70</v>
       </c>
@@ -12122,7 +12272,7 @@
       </c>
       <c r="P80" s="22"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B81" s="20">
         <v>71</v>
       </c>
@@ -12153,7 +12303,7 @@
       </c>
       <c r="P81" s="22"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B82" s="20">
         <v>72</v>
       </c>
@@ -12184,7 +12334,7 @@
       </c>
       <c r="P82" s="22"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B83" s="20">
         <v>73</v>
       </c>
@@ -12215,7 +12365,7 @@
       </c>
       <c r="P83" s="22"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B84" s="20">
         <v>74</v>
       </c>
@@ -12246,7 +12396,7 @@
       </c>
       <c r="P84" s="22"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B85" s="20">
         <v>75</v>
       </c>
@@ -12277,7 +12427,7 @@
       </c>
       <c r="P85" s="22"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B86" s="20">
         <v>76</v>
       </c>
@@ -12308,7 +12458,7 @@
       </c>
       <c r="P86" s="22"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B87" s="20">
         <v>77</v>
       </c>
@@ -12339,7 +12489,7 @@
       </c>
       <c r="P87" s="22"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B88" s="20">
         <v>78</v>
       </c>
@@ -12370,7 +12520,7 @@
       </c>
       <c r="P88" s="22"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B89" s="20">
         <v>79</v>
       </c>
@@ -12401,7 +12551,7 @@
       </c>
       <c r="P89" s="22"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B90" s="20">
         <v>80</v>
       </c>
@@ -12432,7 +12582,7 @@
       </c>
       <c r="P90" s="22"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B91" s="20">
         <v>81</v>
       </c>
@@ -12463,7 +12613,7 @@
       </c>
       <c r="P91" s="22"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B92" s="20">
         <v>82</v>
       </c>
@@ -12494,7 +12644,7 @@
       </c>
       <c r="P92" s="22"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B93" s="20">
         <v>83</v>
       </c>
@@ -12525,7 +12675,7 @@
       </c>
       <c r="P93" s="22"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B94" s="20">
         <v>84</v>
       </c>
@@ -12556,7 +12706,7 @@
       </c>
       <c r="P94" s="22"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B95" s="20">
         <v>85</v>
       </c>
@@ -12587,7 +12737,7 @@
       </c>
       <c r="P95" s="22"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B96" s="20">
         <v>86</v>
       </c>
@@ -12618,7 +12768,7 @@
       </c>
       <c r="P96" s="22"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B97" s="20">
         <v>87</v>
       </c>
@@ -12649,7 +12799,7 @@
       </c>
       <c r="P97" s="22"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B98" s="20">
         <v>88</v>
       </c>
@@ -12680,7 +12830,7 @@
       </c>
       <c r="P98" s="22"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B99" s="20">
         <v>89</v>
       </c>
@@ -12711,7 +12861,7 @@
       </c>
       <c r="P99" s="22"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B100" s="20">
         <v>90</v>
       </c>
@@ -12742,7 +12892,7 @@
       </c>
       <c r="P100" s="22"/>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B101" s="20">
         <v>91</v>
       </c>
@@ -12773,7 +12923,7 @@
       </c>
       <c r="P101" s="22"/>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B102" s="20">
         <v>92</v>
       </c>
@@ -12804,7 +12954,7 @@
       </c>
       <c r="P102" s="22"/>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B103" s="20">
         <v>93</v>
       </c>
@@ -12835,7 +12985,7 @@
       </c>
       <c r="P103" s="22"/>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B104" s="20">
         <v>94</v>
       </c>
@@ -12866,7 +13016,7 @@
       </c>
       <c r="P104" s="22"/>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B105" s="20">
         <v>95</v>
       </c>
@@ -12897,7 +13047,7 @@
       </c>
       <c r="P105" s="22"/>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B106" s="20">
         <v>96</v>
       </c>
@@ -12928,7 +13078,7 @@
       </c>
       <c r="P106" s="22"/>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B107" s="20">
         <v>97</v>
       </c>
@@ -12959,7 +13109,7 @@
       </c>
       <c r="P107" s="22"/>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B108" s="20">
         <v>98</v>
       </c>
@@ -12990,7 +13140,7 @@
       </c>
       <c r="P108" s="22"/>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B109" s="20">
         <v>99</v>
       </c>
@@ -13021,7 +13171,7 @@
       </c>
       <c r="P109" s="22"/>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B110" s="20">
         <v>100</v>
       </c>
@@ -13168,12 +13318,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:J39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B2" s="63" t="s">
         <v>88</v>
       </c>
@@ -13186,7 +13336,7 @@
       <c r="I2" s="63"/>
       <c r="J2" s="63"/>
     </row>
-    <row r="4" spans="2:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="64" t="s">
         <v>89</v>
       </c>
@@ -13199,7 +13349,7 @@
       <c r="I4" s="64"/>
       <c r="J4" s="64"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
       <c r="D5" s="64"/>
@@ -13210,7 +13360,7 @@
       <c r="I5" s="64"/>
       <c r="J5" s="64"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B6" s="64"/>
       <c r="C6" s="64"/>
       <c r="D6" s="64"/>
@@ -13221,7 +13371,7 @@
       <c r="I6" s="64"/>
       <c r="J6" s="64"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
@@ -13232,7 +13382,7 @@
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
         <v>90</v>
       </c>
@@ -13245,7 +13395,7 @@
       <c r="I8" s="30"/>
       <c r="J8" s="30"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B9" s="31" t="s">
         <v>91</v>
       </c>
@@ -13258,7 +13408,7 @@
       <c r="I9" s="30"/>
       <c r="J9" s="30"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B10" s="31" t="s">
         <v>92</v>
       </c>
@@ -13271,7 +13421,7 @@
       <c r="I10" s="30"/>
       <c r="J10" s="30"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B11" s="31" t="s">
         <v>31</v>
       </c>
@@ -13284,7 +13434,7 @@
       <c r="I11" s="30"/>
       <c r="J11" s="30"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B12" s="31" t="s">
         <v>36</v>
       </c>
@@ -13297,7 +13447,7 @@
       <c r="I12" s="30"/>
       <c r="J12" s="30"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B13" s="31" t="s">
         <v>93</v>
       </c>
@@ -13310,7 +13460,7 @@
       <c r="I13" s="30"/>
       <c r="J13" s="30"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B14" s="32" t="s">
         <v>94</v>
       </c>
@@ -13323,7 +13473,7 @@
       <c r="I14" s="30"/>
       <c r="J14" s="30"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B15" s="8"/>
       <c r="C15" s="30"/>
       <c r="D15" s="30"/>
@@ -13334,7 +13484,7 @@
       <c r="I15" s="30"/>
       <c r="J15" s="30"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B16" s="33" t="s">
         <v>95</v>
       </c>
@@ -13347,7 +13497,7 @@
       <c r="I16" s="30"/>
       <c r="J16" s="30"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B17" s="34" t="s">
         <v>96</v>
       </c>
@@ -13360,7 +13510,7 @@
       <c r="I17" s="30"/>
       <c r="J17" s="30"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B18" s="34" t="s">
         <v>97</v>
       </c>
@@ -13373,7 +13523,7 @@
       <c r="I18" s="30"/>
       <c r="J18" s="30"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B19" s="35" t="s">
         <v>98</v>
       </c>
@@ -13386,7 +13536,7 @@
       <c r="I19" s="30"/>
       <c r="J19" s="30"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B20" s="8"/>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
@@ -13397,7 +13547,7 @@
       <c r="I20" s="30"/>
       <c r="J20" s="30"/>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B21" s="33" t="s">
         <v>99</v>
       </c>
@@ -13410,7 +13560,7 @@
       <c r="I21" s="30"/>
       <c r="J21" s="30"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B22" s="36">
         <v>45658</v>
       </c>
@@ -13423,7 +13573,7 @@
       <c r="I22" s="30"/>
       <c r="J22" s="30"/>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B23" s="37">
         <v>46062.354166666701</v>
       </c>
@@ -13436,7 +13586,7 @@
       <c r="I23" s="30"/>
       <c r="J23" s="30"/>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B24" s="30"/>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
@@ -13447,7 +13597,7 @@
       <c r="I24" s="30"/>
       <c r="J24" s="30"/>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B25" s="38" t="s">
         <v>100</v>
       </c>
@@ -13464,7 +13614,7 @@
       <c r="I25" s="40"/>
       <c r="J25" s="41"/>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" s="42" t="s">
         <v>76</v>
       </c>
@@ -13487,7 +13637,7 @@
       <c r="I26" s="30"/>
       <c r="J26" s="44"/>
     </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B27" s="42" t="s">
         <v>45</v>
       </c>
@@ -13514,7 +13664,7 @@
       </c>
       <c r="J27" s="44"/>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B28" s="42" t="s">
         <v>73</v>
       </c>
@@ -13539,7 +13689,7 @@
       <c r="I28" s="30"/>
       <c r="J28" s="44"/>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29" s="42" t="s">
         <v>37</v>
       </c>
@@ -13566,7 +13716,7 @@
       </c>
       <c r="J29" s="44"/>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B30" s="42" t="s">
         <v>56</v>
       </c>
@@ -13593,7 +13743,7 @@
       </c>
       <c r="J30" s="44"/>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B31" s="45" t="s">
         <v>32</v>
       </c>
@@ -13622,7 +13772,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B32" s="46" t="s">
         <v>115</v>
       </c>
@@ -13639,7 +13789,7 @@
       <c r="I32" s="48"/>
       <c r="J32" s="49"/>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B33" s="30"/>
       <c r="C33" s="30"/>
       <c r="D33" s="30"/>
@@ -13650,7 +13800,7 @@
       <c r="I33" s="30"/>
       <c r="J33" s="30"/>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B34" s="50" t="s">
         <v>116</v>
       </c>
@@ -13665,7 +13815,7 @@
       <c r="I34" s="30"/>
       <c r="J34" s="30"/>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B35" s="45" t="s">
         <v>30</v>
       </c>
@@ -13680,7 +13830,7 @@
       <c r="I35" s="30"/>
       <c r="J35" s="30"/>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B36" s="45" t="s">
         <v>35</v>
       </c>
@@ -13695,7 +13845,7 @@
       <c r="I36" s="30"/>
       <c r="J36" s="30"/>
     </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B37" s="45" t="s">
         <v>55</v>
       </c>
@@ -13710,7 +13860,7 @@
       <c r="I37" s="30"/>
       <c r="J37" s="30"/>
     </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B38" s="45" t="s">
         <v>72</v>
       </c>
@@ -13725,7 +13875,7 @@
       <c r="I38" s="30"/>
       <c r="J38" s="30"/>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B39" s="52" t="s">
         <v>115</v>
       </c>

</xml_diff>